<commit_message>
2026 06 15 005
formteaching source tray, target tray panel 생성 수정..
</commit_message>
<xml_diff>
--- a/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
+++ b/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1C2B872-533F-4B59-B667-AB3D7AAE3B56}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481EFD34-D919-417E-A959-652167EB9133}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="8910" windowHeight="10470" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2368,6 +2368,9 @@
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2397,9 +2400,6 @@
     </xf>
     <xf numFmtId="176" fontId="3" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2691,12 +2691,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
     </row>
     <row r="3" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2714,12 +2714,12 @@
       </c>
     </row>
     <row r="5" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="40"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="41"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="42"/>
     </row>
     <row r="6" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="14" t="s">
@@ -2793,12 +2793,12 @@
       <c r="H13" s="13"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="38"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="38"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="39"/>
     </row>
     <row r="17" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="18" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2883,11 +2883,11 @@
       </c>
     </row>
     <row r="3" spans="2:4" ht="25.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="45" t="s">
+      <c r="B3" s="46" t="s">
         <v>620</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="48"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="25" t="s">
@@ -2920,7 +2920,7 @@
       <c r="B7" s="25" t="s">
         <v>624</v>
       </c>
-      <c r="C7" s="48" t="s">
+      <c r="C7" s="38" t="s">
         <v>625</v>
       </c>
       <c r="D7" s="16"/>
@@ -2996,11 +2996,11 @@
       <c r="D21" s="10"/>
     </row>
     <row r="22" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="42" t="s">
+      <c r="B22" s="43" t="s">
         <v>619</v>
       </c>
-      <c r="C22" s="43"/>
-      <c r="D22" s="44"/>
+      <c r="C22" s="44"/>
+      <c r="D22" s="45"/>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B23" s="25"/>

</xml_diff>

<commit_message>
2026 06 15 006
FormTeaching 수정 1차 완료.
</commit_message>
<xml_diff>
--- a/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
+++ b/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481EFD34-D919-417E-A959-652167EB9133}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D122993B-7CEA-4D52-8653-3BEC7791EAC6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="8910" windowHeight="10470" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="626">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="628">
   <si>
     <t>내용</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1953,6 +1953,14 @@
   </si>
   <si>
     <t>mod gripper sorting/Inserting 수정. =&gt; 샘플선별기 참고</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>6/15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>JOG 제어에서 gripper는 몇초간 눌러야 동작하도록 수정. 그리퍼 열기/닫기도 포함</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2926,8 +2934,12 @@
       <c r="D7" s="16"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B8" s="25"/>
-      <c r="C8" s="28"/>
+      <c r="B8" s="25" t="s">
+        <v>626</v>
+      </c>
+      <c r="C8" s="32" t="s">
+        <v>627</v>
+      </c>
       <c r="D8" s="16"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
2026 06 19 001
언어변경 - FormTeaching 수정 중.
</commit_message>
<xml_diff>
--- a/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
+++ b/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D122993B-7CEA-4D52-8653-3BEC7791EAC6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C408EE5-F469-40A6-A464-A449D95D8FCC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="8910" windowHeight="10470" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="628">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="630">
   <si>
     <t>내용</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1961,6 +1961,14 @@
   </si>
   <si>
     <t>JOG 제어에서 gripper는 몇초간 눌러야 동작하도록 수정. 그리퍼 열기/닫기도 포함</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>그리퍼 열기 조건 추가 - 헝가리 불량선별기 참고.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>6/18</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2943,8 +2951,12 @@
       <c r="D8" s="16"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B9" s="25"/>
-      <c r="C9" s="32"/>
+      <c r="B9" s="25" t="s">
+        <v>629</v>
+      </c>
+      <c r="C9" s="32" t="s">
+        <v>628</v>
+      </c>
       <c r="D9" s="10"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
2026 06 26 001
Form Interface 수정 중.
</commit_message>
<xml_diff>
--- a/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
+++ b/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C408EE5-F469-40A6-A464-A449D95D8FCC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99469ACE-BBAD-4DA4-B7AD-6AA0245A86A9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="8910" windowHeight="10470" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="630">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="632">
   <si>
     <t>내용</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1969,6 +1969,15 @@
   </si>
   <si>
     <t>6/18</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>6/25</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>트레이 바코드 리딩후 FMS에 보고. Tray info 받아서 파일저장. 에러 발생시 다시 바코드 읽고  tray info 받았을 때 저장된 내용과 일치하는지 확인. 
+-&gt; 셀 1개 이재시마다 파일저장 업데이트 필요</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2959,9 +2968,13 @@
       </c>
       <c r="D9" s="10"/>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B10" s="25"/>
-      <c r="C10" s="18"/>
+    <row r="10" spans="2:4" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="B10" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C10" s="32" t="s">
+        <v>631</v>
+      </c>
       <c r="D10" s="17"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
2026 07 23 001
1. 연기감지기 연결
2. 바코드리더기 연결
3. fms 추가.
</commit_message>
<xml_diff>
--- a/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
+++ b/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99469ACE-BBAD-4DA4-B7AD-6AA0245A86A9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5538BC5B-0A15-467D-8B26-0DDB076D5887}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="8910" windowHeight="10470" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="632">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="636">
   <si>
     <t>내용</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1978,6 +1978,22 @@
   <si>
     <t>트레이 바코드 리딩후 FMS에 보고. Tray info 받아서 파일저장. 에러 발생시 다시 바코드 읽고  tray info 받았을 때 저장된 내용과 일치하는지 확인. 
 -&gt; 셀 1개 이재시마다 파일저장 업데이트 필요</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>6/29</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>바코드리더 CommRxFlag에서 유효성 검사 보완필요</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>7/8</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>선별트레이 바코드 스캔하고 상위에서 데이터 받는 부분 문의 =&gt; FMS</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1989,7 +2005,7 @@
     <numFmt numFmtId="176" formatCode="mm&quot;월&quot;\ dd&quot;일&quot;"/>
     <numFmt numFmtId="177" formatCode="&quot;₩&quot;#,##0"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2030,23 +2046,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <strike/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="3"/>
-      <charset val="129"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <strike/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <strike/>
       <sz val="11"/>
@@ -2057,10 +2056,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <strike/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
@@ -2308,7 +2305,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -2337,9 +2334,6 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2351,37 +2345,13 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2390,11 +2360,6 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2425,6 +2390,48 @@
     </xf>
     <xf numFmtId="176" fontId="3" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2716,12 +2723,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
     </row>
     <row r="3" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2739,68 +2746,68 @@
       </c>
     </row>
     <row r="5" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="40" t="s">
+      <c r="B5" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
-      <c r="E5" s="42"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="26"/>
     </row>
     <row r="6" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="E6" s="14" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
     </row>
     <row r="8" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
     </row>
     <row r="9" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
     </row>
     <row r="10" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="E10" s="14" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2815,15 +2822,15 @@
       <c r="E11" s="7"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="H13" s="13"/>
+      <c r="H13" s="12"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="39" t="s">
+      <c r="B16" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="39"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
     </row>
     <row r="17" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="18" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2890,17 +2897,17 @@
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
-    <col min="2" max="2" width="9.875" style="33" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="102.375" style="8" customWidth="1"/>
+    <col min="2" max="2" width="9.875" style="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="102.375" style="33" customWidth="1"/>
     <col min="4" max="4" width="68.625" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="21" t="s">
         <v>618</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="34" t="s">
         <v>0</v>
       </c>
       <c r="D2" s="9" t="s">
@@ -2908,480 +2915,488 @@
       </c>
     </row>
     <row r="3" spans="2:4" ht="25.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="30" t="s">
         <v>620</v>
       </c>
-      <c r="C3" s="47"/>
-      <c r="D3" s="48"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="32"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="18" t="s">
         <v>617</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="46" t="s">
         <v>621</v>
       </c>
       <c r="D4" s="10"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="18" t="s">
         <v>617</v>
       </c>
-      <c r="C5" s="37" t="s">
+      <c r="C5" s="35" t="s">
         <v>622</v>
       </c>
       <c r="D5" s="10"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="18" t="s">
         <v>617</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="C6" s="42" t="s">
         <v>623</v>
       </c>
-      <c r="D6" s="16"/>
+      <c r="D6" s="15"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="18" t="s">
         <v>624</v>
       </c>
-      <c r="C7" s="38" t="s">
+      <c r="C7" s="37" t="s">
         <v>625</v>
       </c>
-      <c r="D7" s="16"/>
+      <c r="D7" s="15"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="18" t="s">
         <v>626</v>
       </c>
-      <c r="C8" s="32" t="s">
+      <c r="C8" s="36" t="s">
         <v>627</v>
       </c>
-      <c r="D8" s="16"/>
+      <c r="D8" s="15"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="18" t="s">
         <v>629</v>
       </c>
-      <c r="C9" s="32" t="s">
+      <c r="C9" s="36" t="s">
         <v>628</v>
       </c>
       <c r="D9" s="10"/>
     </row>
     <row r="10" spans="2:4" ht="49.5" x14ac:dyDescent="0.3">
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="18" t="s">
         <v>630</v>
       </c>
-      <c r="C10" s="32" t="s">
+      <c r="C10" s="36" t="s">
         <v>631</v>
       </c>
-      <c r="D10" s="17"/>
+      <c r="D10" s="16"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B11" s="25"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="16"/>
+      <c r="B11" s="18" t="s">
+        <v>632</v>
+      </c>
+      <c r="C11" s="36" t="s">
+        <v>633</v>
+      </c>
+      <c r="D11" s="15"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B12" s="25"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="16"/>
+      <c r="B12" s="18" t="s">
+        <v>634</v>
+      </c>
+      <c r="C12" s="36" t="s">
+        <v>635</v>
+      </c>
+      <c r="D12" s="15"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="25"/>
-      <c r="C13" s="28"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="37"/>
       <c r="D13" s="10"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="25"/>
-      <c r="C14" s="18"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="38"/>
       <c r="D14" s="10"/>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B15" s="25"/>
-      <c r="C15" s="19"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="39"/>
       <c r="D15" s="10"/>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B16" s="25"/>
-      <c r="C16" s="19"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="39"/>
       <c r="D16" s="10"/>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="25"/>
-      <c r="C17" s="20"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="40"/>
       <c r="D17" s="10"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="25"/>
-      <c r="C18" s="20"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="40"/>
       <c r="D18" s="10"/>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B19" s="25"/>
-      <c r="C19" s="21"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="40"/>
       <c r="D19" s="10"/>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B20" s="25"/>
-      <c r="C20" s="19"/>
+      <c r="B20" s="18"/>
+      <c r="C20" s="39"/>
       <c r="D20" s="10"/>
     </row>
     <row r="21" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="25"/>
-      <c r="C21" s="26"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="41"/>
       <c r="D21" s="10"/>
     </row>
     <row r="22" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="43" t="s">
+      <c r="B22" s="27" t="s">
         <v>619</v>
       </c>
-      <c r="C22" s="44"/>
-      <c r="D22" s="45"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="29"/>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B23" s="25"/>
-      <c r="C23" s="30"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="43"/>
       <c r="D23" s="10"/>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B24" s="25"/>
-      <c r="C24" s="27"/>
+      <c r="B24" s="18"/>
+      <c r="C24" s="44"/>
       <c r="D24" s="10"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B25" s="25"/>
-      <c r="C25" s="30"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="43"/>
       <c r="D25" s="10"/>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B26" s="25"/>
-      <c r="C26" s="27"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="44"/>
       <c r="D26" s="10"/>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B27" s="25"/>
-      <c r="C27" s="27"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="44"/>
       <c r="D27" s="10"/>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B28" s="25"/>
-      <c r="C28" s="27"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="44"/>
       <c r="D28" s="10"/>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B29" s="25"/>
-      <c r="C29" s="27"/>
+      <c r="B29" s="18"/>
+      <c r="C29" s="44"/>
       <c r="D29" s="10"/>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B30" s="25"/>
-      <c r="C30" s="27"/>
+      <c r="B30" s="18"/>
+      <c r="C30" s="44"/>
       <c r="D30" s="10"/>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B31" s="25"/>
-      <c r="C31" s="27"/>
+      <c r="B31" s="18"/>
+      <c r="C31" s="44"/>
       <c r="D31" s="10"/>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B32" s="25"/>
-      <c r="C32" s="27"/>
+      <c r="B32" s="18"/>
+      <c r="C32" s="44"/>
       <c r="D32" s="10"/>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B33" s="25"/>
-      <c r="C33" s="27"/>
+      <c r="B33" s="18"/>
+      <c r="C33" s="44"/>
       <c r="D33" s="10"/>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B34" s="25"/>
-      <c r="C34" s="27"/>
+      <c r="B34" s="18"/>
+      <c r="C34" s="44"/>
       <c r="D34" s="10"/>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B35" s="25"/>
-      <c r="C35" s="27"/>
+      <c r="B35" s="18"/>
+      <c r="C35" s="44"/>
       <c r="D35" s="10"/>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B36" s="25"/>
-      <c r="C36" s="27"/>
+      <c r="B36" s="18"/>
+      <c r="C36" s="44"/>
       <c r="D36" s="10"/>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B37" s="25"/>
-      <c r="C37" s="30"/>
+      <c r="B37" s="18"/>
+      <c r="C37" s="43"/>
       <c r="D37" s="10"/>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B38" s="25"/>
-      <c r="C38" s="30"/>
+      <c r="B38" s="18"/>
+      <c r="C38" s="43"/>
       <c r="D38" s="10"/>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B39" s="25"/>
-      <c r="C39" s="30"/>
+      <c r="B39" s="18"/>
+      <c r="C39" s="43"/>
       <c r="D39" s="10"/>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B40" s="25"/>
-      <c r="C40" s="27"/>
+      <c r="B40" s="18"/>
+      <c r="C40" s="44"/>
       <c r="D40" s="10"/>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B41" s="25"/>
-      <c r="C41" s="27"/>
+      <c r="B41" s="18"/>
+      <c r="C41" s="44"/>
       <c r="D41" s="10"/>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B42" s="25"/>
-      <c r="C42" s="30"/>
+      <c r="B42" s="18"/>
+      <c r="C42" s="43"/>
       <c r="D42" s="10"/>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B43" s="25"/>
-      <c r="C43" s="27"/>
+      <c r="B43" s="18"/>
+      <c r="C43" s="44"/>
       <c r="D43" s="10"/>
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B44" s="25"/>
-      <c r="C44" s="20"/>
+      <c r="B44" s="18"/>
+      <c r="C44" s="40"/>
       <c r="D44" s="10"/>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B45" s="25"/>
-      <c r="C45" s="20"/>
+      <c r="B45" s="18"/>
+      <c r="C45" s="40"/>
       <c r="D45" s="10"/>
     </row>
     <row r="46" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B46" s="25"/>
-      <c r="C46" s="27"/>
+      <c r="B46" s="18"/>
+      <c r="C46" s="44"/>
       <c r="D46" s="10"/>
     </row>
     <row r="47" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B47" s="25"/>
-      <c r="C47" s="27"/>
+      <c r="B47" s="18"/>
+      <c r="C47" s="44"/>
       <c r="D47" s="10"/>
     </row>
     <row r="48" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B48" s="25"/>
-      <c r="C48" s="27"/>
+      <c r="B48" s="18"/>
+      <c r="C48" s="44"/>
       <c r="D48" s="10"/>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B49" s="25"/>
-      <c r="C49" s="27"/>
+      <c r="B49" s="18"/>
+      <c r="C49" s="44"/>
       <c r="D49" s="10"/>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B50" s="25"/>
-      <c r="C50" s="27"/>
+      <c r="B50" s="18"/>
+      <c r="C50" s="44"/>
       <c r="D50" s="10"/>
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B51" s="25"/>
-      <c r="C51" s="27"/>
+      <c r="B51" s="18"/>
+      <c r="C51" s="44"/>
       <c r="D51" s="10"/>
     </row>
     <row r="52" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B52" s="25"/>
-      <c r="C52" s="27"/>
+      <c r="B52" s="18"/>
+      <c r="C52" s="44"/>
       <c r="D52" s="10"/>
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B53" s="25"/>
-      <c r="C53" s="20"/>
+      <c r="B53" s="18"/>
+      <c r="C53" s="40"/>
       <c r="D53" s="10"/>
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B54" s="25"/>
-      <c r="C54" s="27"/>
+      <c r="B54" s="18"/>
+      <c r="C54" s="44"/>
       <c r="D54" s="10"/>
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B55" s="25"/>
-      <c r="C55" s="30"/>
+      <c r="B55" s="18"/>
+      <c r="C55" s="43"/>
       <c r="D55" s="10"/>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B56" s="25"/>
-      <c r="C56" s="20"/>
+      <c r="B56" s="18"/>
+      <c r="C56" s="40"/>
       <c r="D56" s="10"/>
     </row>
     <row r="57" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B57" s="25"/>
-      <c r="C57" s="27"/>
+      <c r="B57" s="18"/>
+      <c r="C57" s="44"/>
       <c r="D57" s="10"/>
     </row>
     <row r="58" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B58" s="25"/>
-      <c r="C58" s="20"/>
+      <c r="B58" s="18"/>
+      <c r="C58" s="40"/>
       <c r="D58" s="10"/>
     </row>
     <row r="59" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B59" s="25"/>
-      <c r="C59" s="20"/>
+      <c r="B59" s="18"/>
+      <c r="C59" s="40"/>
       <c r="D59" s="10"/>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B60" s="25"/>
-      <c r="C60" s="19"/>
+      <c r="B60" s="18"/>
+      <c r="C60" s="39"/>
       <c r="D60" s="10"/>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B61" s="25"/>
-      <c r="C61" s="28"/>
-      <c r="D61" s="24"/>
+      <c r="B61" s="18"/>
+      <c r="C61" s="37"/>
+      <c r="D61" s="17"/>
     </row>
     <row r="62" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B62" s="25"/>
-      <c r="C62" s="27"/>
+      <c r="B62" s="18"/>
+      <c r="C62" s="44"/>
       <c r="D62" s="10"/>
     </row>
     <row r="63" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B63" s="25"/>
-      <c r="C63" s="27"/>
+      <c r="B63" s="18"/>
+      <c r="C63" s="44"/>
       <c r="D63" s="10"/>
     </row>
     <row r="64" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B64" s="25"/>
-      <c r="C64" s="27"/>
+      <c r="B64" s="18"/>
+      <c r="C64" s="44"/>
       <c r="D64" s="10"/>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B65" s="25"/>
-      <c r="C65" s="27"/>
+      <c r="B65" s="18"/>
+      <c r="C65" s="44"/>
       <c r="D65" s="10"/>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B66" s="25"/>
-      <c r="C66" s="27"/>
+      <c r="B66" s="18"/>
+      <c r="C66" s="44"/>
       <c r="D66" s="10"/>
     </row>
     <row r="67" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B67" s="25"/>
-      <c r="C67" s="28"/>
+      <c r="B67" s="18"/>
+      <c r="C67" s="37"/>
       <c r="D67" s="10"/>
     </row>
     <row r="68" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B68" s="25"/>
-      <c r="C68" s="27"/>
+      <c r="B68" s="18"/>
+      <c r="C68" s="44"/>
       <c r="D68" s="10"/>
     </row>
     <row r="69" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B69" s="25"/>
-      <c r="C69" s="28"/>
+      <c r="B69" s="18"/>
+      <c r="C69" s="37"/>
       <c r="D69" s="10"/>
     </row>
     <row r="70" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B70" s="25"/>
-      <c r="C70" s="30"/>
+      <c r="B70" s="18"/>
+      <c r="C70" s="43"/>
       <c r="D70" s="10"/>
     </row>
     <row r="71" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B71" s="25"/>
-      <c r="C71" s="30"/>
+      <c r="B71" s="18"/>
+      <c r="C71" s="43"/>
       <c r="D71" s="10"/>
     </row>
     <row r="72" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B72" s="25"/>
-      <c r="C72" s="28"/>
+      <c r="B72" s="18"/>
+      <c r="C72" s="37"/>
       <c r="D72" s="10"/>
     </row>
     <row r="73" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B73" s="25"/>
-      <c r="C73" s="28"/>
+      <c r="B73" s="18"/>
+      <c r="C73" s="37"/>
       <c r="D73" s="10"/>
     </row>
     <row r="74" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B74" s="25"/>
-      <c r="C74" s="28"/>
+      <c r="B74" s="18"/>
+      <c r="C74" s="37"/>
       <c r="D74" s="10"/>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B75" s="25"/>
-      <c r="C75" s="28"/>
+      <c r="B75" s="18"/>
+      <c r="C75" s="37"/>
       <c r="D75" s="10"/>
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B76" s="25"/>
-      <c r="C76" s="28"/>
+      <c r="B76" s="18"/>
+      <c r="C76" s="37"/>
       <c r="D76" s="10"/>
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B77" s="25"/>
-      <c r="C77" s="28"/>
+      <c r="B77" s="18"/>
+      <c r="C77" s="37"/>
       <c r="D77" s="10"/>
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B78" s="25"/>
-      <c r="C78" s="28"/>
+      <c r="B78" s="18"/>
+      <c r="C78" s="37"/>
       <c r="D78" s="10"/>
     </row>
     <row r="79" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B79" s="25"/>
-      <c r="C79" s="28"/>
+      <c r="B79" s="18"/>
+      <c r="C79" s="37"/>
       <c r="D79" s="10"/>
     </row>
     <row r="80" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B80" s="25"/>
-      <c r="C80" s="28"/>
+      <c r="B80" s="18"/>
+      <c r="C80" s="37"/>
       <c r="D80" s="10"/>
     </row>
     <row r="81" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B81" s="25"/>
-      <c r="C81" s="28"/>
+      <c r="B81" s="18"/>
+      <c r="C81" s="37"/>
       <c r="D81" s="10"/>
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B82" s="25"/>
-      <c r="C82" s="32"/>
+      <c r="B82" s="18"/>
+      <c r="C82" s="36"/>
       <c r="D82" s="10"/>
     </row>
     <row r="83" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B83" s="25"/>
-      <c r="C83" s="32"/>
+      <c r="B83" s="18"/>
+      <c r="C83" s="36"/>
       <c r="D83" s="10"/>
     </row>
     <row r="84" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B84" s="25"/>
-      <c r="C84" s="32"/>
+      <c r="B84" s="18"/>
+      <c r="C84" s="36"/>
       <c r="D84" s="10"/>
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B85" s="25"/>
-      <c r="C85" s="26"/>
+      <c r="B85" s="18"/>
+      <c r="C85" s="41"/>
       <c r="D85" s="10"/>
     </row>
     <row r="86" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B86" s="25"/>
-      <c r="C86" s="26"/>
+      <c r="B86" s="18"/>
+      <c r="C86" s="41"/>
       <c r="D86" s="10"/>
     </row>
     <row r="87" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B87" s="25"/>
-      <c r="C87" s="26"/>
+      <c r="B87" s="18"/>
+      <c r="C87" s="41"/>
       <c r="D87" s="10"/>
     </row>
     <row r="88" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B88" s="25"/>
-      <c r="C88" s="26"/>
+      <c r="B88" s="18"/>
+      <c r="C88" s="41"/>
       <c r="D88" s="10"/>
     </row>
     <row r="89" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B89" s="25"/>
-      <c r="C89" s="22"/>
+      <c r="B89" s="18"/>
+      <c r="C89" s="40"/>
       <c r="D89" s="10"/>
     </row>
     <row r="90" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B90" s="25"/>
-      <c r="C90" s="22"/>
+      <c r="B90" s="18"/>
+      <c r="C90" s="40"/>
       <c r="D90" s="10"/>
     </row>
     <row r="91" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B91" s="35"/>
-      <c r="C91" s="23"/>
+      <c r="B91" s="22"/>
+      <c r="C91" s="45"/>
       <c r="D91" s="11"/>
     </row>
   </sheetData>
@@ -15682,34 +15697,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" s="29"/>
+      <c r="A1" s="19"/>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="29"/>
+      <c r="A2" s="19"/>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="29"/>
+      <c r="A3" s="19"/>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="29"/>
+      <c r="A4" s="19"/>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="29"/>
+      <c r="A5" s="19"/>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" s="29"/>
+      <c r="A6" s="19"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" s="29"/>
+      <c r="A7" s="19"/>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" s="29"/>
+      <c r="A8" s="19"/>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" s="29"/>
+      <c r="A9" s="19"/>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" s="29"/>
+      <c r="A10" s="19"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
2026 09 10 001
- z축 속도 수정. 80%, 20% 다르게.
- 힌디어 선택 숨김.
</commit_message>
<xml_diff>
--- a/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
+++ b/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5538BC5B-0A15-467D-8B26-0DDB076D5887}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58DAE065-B991-4603-BE81-EDC3BC7CB7AC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="8910" windowHeight="10470" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="636">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="644">
   <si>
     <t>내용</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1994,6 +1994,38 @@
   </si>
   <si>
     <t>선별트레이 바코드 스캔하고 상위에서 데이터 받는 부분 문의 =&gt; FMS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>9/10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>검수</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fms 알람 발생시 설비 알람 표시 -&gt; fms 알람 해제시 설비 알람 해제.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>티칭값 저장시 암호입력.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>티칭값 저장시 도면치수 참고하여 오차범위 내에서만 가능 (10 mm 이내)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>불량트레이 일정 수량 초과시 트레이 아웃 경고</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>buffer overflow 에러시 서보 멈춤 동작 - pc 제어인지 서보 셋팅인지 확인. =&gt; 멈춤 코드 있음. 속도가 빨라서 늦은것 같음.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>z축 속도 별도 셋팅. 80% 속도, 20% 속도</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2005,7 +2037,7 @@
     <numFmt numFmtId="176" formatCode="mm&quot;월&quot;\ dd&quot;일&quot;"/>
     <numFmt numFmtId="177" formatCode="&quot;₩&quot;#,##0"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2058,6 +2090,32 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
       <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
@@ -2305,7 +2363,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -2361,43 +2419,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2432,6 +2457,48 @@
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2723,12 +2790,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
     </row>
     <row r="3" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2746,12 +2813,12 @@
       </c>
     </row>
     <row r="5" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="26"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="39"/>
     </row>
     <row r="6" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="13" t="s">
@@ -2825,12 +2892,12 @@
       <c r="H13" s="12"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
+      <c r="C16" s="36"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="36"/>
     </row>
     <row r="17" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="18" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2893,12 +2960,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B66418C2-2F25-4DF5-AD93-3985FBAF3208}">
-  <dimension ref="B1:D91"/>
+  <dimension ref="B1:D98"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="9.875" style="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="102.375" style="33" customWidth="1"/>
+    <col min="3" max="3" width="102.375" style="23" customWidth="1"/>
     <col min="4" max="4" width="68.625" style="8" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2907,7 +2974,7 @@
       <c r="B2" s="21" t="s">
         <v>618</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="C2" s="24" t="s">
         <v>0</v>
       </c>
       <c r="D2" s="9" t="s">
@@ -2915,17 +2982,17 @@
       </c>
     </row>
     <row r="3" spans="2:4" ht="25.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="43" t="s">
         <v>620</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="32"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="45"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="18" t="s">
         <v>617</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="35" t="s">
         <v>621</v>
       </c>
       <c r="D4" s="10"/>
@@ -2934,7 +3001,7 @@
       <c r="B5" s="18" t="s">
         <v>617</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="C5" s="46" t="s">
         <v>622</v>
       </c>
       <c r="D5" s="10"/>
@@ -2943,7 +3010,7 @@
       <c r="B6" s="18" t="s">
         <v>617</v>
       </c>
-      <c r="C6" s="42" t="s">
+      <c r="C6" s="31" t="s">
         <v>623</v>
       </c>
       <c r="D6" s="15"/>
@@ -2952,7 +3019,7 @@
       <c r="B7" s="18" t="s">
         <v>624</v>
       </c>
-      <c r="C7" s="37" t="s">
+      <c r="C7" s="26" t="s">
         <v>625</v>
       </c>
       <c r="D7" s="15"/>
@@ -2961,7 +3028,7 @@
       <c r="B8" s="18" t="s">
         <v>626</v>
       </c>
-      <c r="C8" s="36" t="s">
+      <c r="C8" s="31" t="s">
         <v>627</v>
       </c>
       <c r="D8" s="15"/>
@@ -2970,7 +3037,7 @@
       <c r="B9" s="18" t="s">
         <v>629</v>
       </c>
-      <c r="C9" s="36" t="s">
+      <c r="C9" s="31" t="s">
         <v>628</v>
       </c>
       <c r="D9" s="10"/>
@@ -2979,7 +3046,7 @@
       <c r="B10" s="18" t="s">
         <v>630</v>
       </c>
-      <c r="C10" s="36" t="s">
+      <c r="C10" s="31" t="s">
         <v>631</v>
       </c>
       <c r="D10" s="16"/>
@@ -2988,7 +3055,7 @@
       <c r="B11" s="18" t="s">
         <v>632</v>
       </c>
-      <c r="C11" s="36" t="s">
+      <c r="C11" s="31" t="s">
         <v>633</v>
       </c>
       <c r="D11" s="15"/>
@@ -2997,411 +3064,472 @@
       <c r="B12" s="18" t="s">
         <v>634</v>
       </c>
-      <c r="C12" s="36" t="s">
+      <c r="C12" s="31" t="s">
         <v>635</v>
       </c>
       <c r="D12" s="15"/>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:4" ht="26.25" x14ac:dyDescent="0.3">
       <c r="B13" s="18"/>
-      <c r="C13" s="37"/>
+      <c r="C13" s="49" t="s">
+        <v>637</v>
+      </c>
       <c r="D13" s="10"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="18"/>
-      <c r="C14" s="38"/>
+      <c r="B14" s="18" t="s">
+        <v>636</v>
+      </c>
+      <c r="C14" s="47" t="s">
+        <v>638</v>
+      </c>
       <c r="D14" s="10"/>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B15" s="18"/>
-      <c r="C15" s="39"/>
+      <c r="B15" s="18" t="s">
+        <v>636</v>
+      </c>
+      <c r="C15" s="47" t="s">
+        <v>639</v>
+      </c>
       <c r="D15" s="10"/>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B16" s="18"/>
-      <c r="C16" s="39"/>
+      <c r="B16" s="18" t="s">
+        <v>636</v>
+      </c>
+      <c r="C16" s="47" t="s">
+        <v>640</v>
+      </c>
       <c r="D16" s="10"/>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="18"/>
-      <c r="C17" s="40"/>
+    <row r="17" spans="2:4" ht="33" x14ac:dyDescent="0.3">
+      <c r="B17" s="18" t="s">
+        <v>636</v>
+      </c>
+      <c r="C17" s="48" t="s">
+        <v>642</v>
+      </c>
       <c r="D17" s="10"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="18"/>
-      <c r="C18" s="40"/>
+      <c r="B18" s="18" t="s">
+        <v>636</v>
+      </c>
+      <c r="C18" s="47" t="s">
+        <v>641</v>
+      </c>
       <c r="D18" s="10"/>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B19" s="18"/>
-      <c r="C19" s="40"/>
+      <c r="B19" s="18" t="s">
+        <v>636</v>
+      </c>
+      <c r="C19" s="47" t="s">
+        <v>643</v>
+      </c>
       <c r="D19" s="10"/>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B20" s="18"/>
-      <c r="C20" s="39"/>
+      <c r="C20" s="27"/>
       <c r="D20" s="10"/>
     </row>
-    <row r="21" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B21" s="18"/>
-      <c r="C21" s="41"/>
+      <c r="C21" s="27"/>
       <c r="D21" s="10"/>
     </row>
-    <row r="22" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="27" t="s">
-        <v>619</v>
-      </c>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B22" s="18"/>
       <c r="C22" s="28"/>
-      <c r="D22" s="29"/>
+      <c r="D22" s="10"/>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B23" s="18"/>
-      <c r="C23" s="43"/>
+      <c r="C23" s="28"/>
       <c r="D23" s="10"/>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B24" s="18"/>
-      <c r="C24" s="44"/>
+      <c r="C24" s="29"/>
       <c r="D24" s="10"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B25" s="18"/>
-      <c r="C25" s="43"/>
+      <c r="C25" s="29"/>
       <c r="D25" s="10"/>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B26" s="18"/>
-      <c r="C26" s="44"/>
+      <c r="C26" s="29"/>
       <c r="D26" s="10"/>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B27" s="18"/>
-      <c r="C27" s="44"/>
+      <c r="C27" s="28"/>
       <c r="D27" s="10"/>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" s="18"/>
-      <c r="C28" s="44"/>
+      <c r="C28" s="30"/>
       <c r="D28" s="10"/>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B29" s="18"/>
-      <c r="C29" s="44"/>
-      <c r="D29" s="10"/>
+    <row r="29" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B29" s="40" t="s">
+        <v>619</v>
+      </c>
+      <c r="C29" s="41"/>
+      <c r="D29" s="42"/>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B30" s="18"/>
-      <c r="C30" s="44"/>
+      <c r="C30" s="32"/>
       <c r="D30" s="10"/>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B31" s="18"/>
-      <c r="C31" s="44"/>
+      <c r="C31" s="33"/>
       <c r="D31" s="10"/>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B32" s="18"/>
-      <c r="C32" s="44"/>
+      <c r="C32" s="32"/>
       <c r="D32" s="10"/>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B33" s="18"/>
-      <c r="C33" s="44"/>
+      <c r="C33" s="33"/>
       <c r="D33" s="10"/>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B34" s="18"/>
-      <c r="C34" s="44"/>
+      <c r="C34" s="33"/>
       <c r="D34" s="10"/>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B35" s="18"/>
-      <c r="C35" s="44"/>
+      <c r="C35" s="33"/>
       <c r="D35" s="10"/>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B36" s="18"/>
-      <c r="C36" s="44"/>
+      <c r="C36" s="33"/>
       <c r="D36" s="10"/>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B37" s="18"/>
-      <c r="C37" s="43"/>
+      <c r="C37" s="33"/>
       <c r="D37" s="10"/>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B38" s="18"/>
-      <c r="C38" s="43"/>
+      <c r="C38" s="33"/>
       <c r="D38" s="10"/>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B39" s="18"/>
-      <c r="C39" s="43"/>
+      <c r="C39" s="33"/>
       <c r="D39" s="10"/>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B40" s="18"/>
-      <c r="C40" s="44"/>
+      <c r="C40" s="33"/>
       <c r="D40" s="10"/>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B41" s="18"/>
-      <c r="C41" s="44"/>
+      <c r="C41" s="33"/>
       <c r="D41" s="10"/>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B42" s="18"/>
-      <c r="C42" s="43"/>
+      <c r="C42" s="33"/>
       <c r="D42" s="10"/>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B43" s="18"/>
-      <c r="C43" s="44"/>
+      <c r="C43" s="33"/>
       <c r="D43" s="10"/>
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B44" s="18"/>
-      <c r="C44" s="40"/>
+      <c r="C44" s="32"/>
       <c r="D44" s="10"/>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B45" s="18"/>
-      <c r="C45" s="40"/>
+      <c r="C45" s="32"/>
       <c r="D45" s="10"/>
     </row>
     <row r="46" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B46" s="18"/>
-      <c r="C46" s="44"/>
+      <c r="C46" s="32"/>
       <c r="D46" s="10"/>
     </row>
     <row r="47" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B47" s="18"/>
-      <c r="C47" s="44"/>
+      <c r="C47" s="33"/>
       <c r="D47" s="10"/>
     </row>
     <row r="48" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B48" s="18"/>
-      <c r="C48" s="44"/>
+      <c r="C48" s="33"/>
       <c r="D48" s="10"/>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B49" s="18"/>
-      <c r="C49" s="44"/>
+      <c r="C49" s="32"/>
       <c r="D49" s="10"/>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B50" s="18"/>
-      <c r="C50" s="44"/>
+      <c r="C50" s="33"/>
       <c r="D50" s="10"/>
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B51" s="18"/>
-      <c r="C51" s="44"/>
+      <c r="C51" s="29"/>
       <c r="D51" s="10"/>
     </row>
     <row r="52" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B52" s="18"/>
-      <c r="C52" s="44"/>
+      <c r="C52" s="29"/>
       <c r="D52" s="10"/>
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B53" s="18"/>
-      <c r="C53" s="40"/>
+      <c r="C53" s="33"/>
       <c r="D53" s="10"/>
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B54" s="18"/>
-      <c r="C54" s="44"/>
+      <c r="C54" s="33"/>
       <c r="D54" s="10"/>
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B55" s="18"/>
-      <c r="C55" s="43"/>
+      <c r="C55" s="33"/>
       <c r="D55" s="10"/>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B56" s="18"/>
-      <c r="C56" s="40"/>
+      <c r="C56" s="33"/>
       <c r="D56" s="10"/>
     </row>
     <row r="57" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B57" s="18"/>
-      <c r="C57" s="44"/>
+      <c r="C57" s="33"/>
       <c r="D57" s="10"/>
     </row>
     <row r="58" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B58" s="18"/>
-      <c r="C58" s="40"/>
+      <c r="C58" s="33"/>
       <c r="D58" s="10"/>
     </row>
     <row r="59" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B59" s="18"/>
-      <c r="C59" s="40"/>
+      <c r="C59" s="33"/>
       <c r="D59" s="10"/>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B60" s="18"/>
-      <c r="C60" s="39"/>
+      <c r="C60" s="29"/>
       <c r="D60" s="10"/>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B61" s="18"/>
-      <c r="C61" s="37"/>
-      <c r="D61" s="17"/>
+      <c r="C61" s="33"/>
+      <c r="D61" s="10"/>
     </row>
     <row r="62" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B62" s="18"/>
-      <c r="C62" s="44"/>
+      <c r="C62" s="32"/>
       <c r="D62" s="10"/>
     </row>
     <row r="63" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B63" s="18"/>
-      <c r="C63" s="44"/>
+      <c r="C63" s="29"/>
       <c r="D63" s="10"/>
     </row>
     <row r="64" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B64" s="18"/>
-      <c r="C64" s="44"/>
+      <c r="C64" s="33"/>
       <c r="D64" s="10"/>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B65" s="18"/>
-      <c r="C65" s="44"/>
+      <c r="C65" s="29"/>
       <c r="D65" s="10"/>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B66" s="18"/>
-      <c r="C66" s="44"/>
+      <c r="C66" s="29"/>
       <c r="D66" s="10"/>
     </row>
     <row r="67" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B67" s="18"/>
-      <c r="C67" s="37"/>
+      <c r="C67" s="28"/>
       <c r="D67" s="10"/>
     </row>
     <row r="68" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B68" s="18"/>
-      <c r="C68" s="44"/>
-      <c r="D68" s="10"/>
+      <c r="C68" s="26"/>
+      <c r="D68" s="17"/>
     </row>
     <row r="69" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B69" s="18"/>
-      <c r="C69" s="37"/>
+      <c r="C69" s="33"/>
       <c r="D69" s="10"/>
     </row>
     <row r="70" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B70" s="18"/>
-      <c r="C70" s="43"/>
+      <c r="C70" s="33"/>
       <c r="D70" s="10"/>
     </row>
     <row r="71" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B71" s="18"/>
-      <c r="C71" s="43"/>
+      <c r="C71" s="33"/>
       <c r="D71" s="10"/>
     </row>
     <row r="72" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B72" s="18"/>
-      <c r="C72" s="37"/>
+      <c r="C72" s="33"/>
       <c r="D72" s="10"/>
     </row>
     <row r="73" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B73" s="18"/>
-      <c r="C73" s="37"/>
+      <c r="C73" s="33"/>
       <c r="D73" s="10"/>
     </row>
     <row r="74" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B74" s="18"/>
-      <c r="C74" s="37"/>
+      <c r="C74" s="26"/>
       <c r="D74" s="10"/>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B75" s="18"/>
-      <c r="C75" s="37"/>
+      <c r="C75" s="33"/>
       <c r="D75" s="10"/>
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B76" s="18"/>
-      <c r="C76" s="37"/>
+      <c r="C76" s="26"/>
       <c r="D76" s="10"/>
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B77" s="18"/>
-      <c r="C77" s="37"/>
+      <c r="C77" s="32"/>
       <c r="D77" s="10"/>
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B78" s="18"/>
-      <c r="C78" s="37"/>
+      <c r="C78" s="32"/>
       <c r="D78" s="10"/>
     </row>
     <row r="79" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B79" s="18"/>
-      <c r="C79" s="37"/>
+      <c r="C79" s="26"/>
       <c r="D79" s="10"/>
     </row>
     <row r="80" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B80" s="18"/>
-      <c r="C80" s="37"/>
+      <c r="C80" s="26"/>
       <c r="D80" s="10"/>
     </row>
     <row r="81" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B81" s="18"/>
-      <c r="C81" s="37"/>
+      <c r="C81" s="26"/>
       <c r="D81" s="10"/>
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B82" s="18"/>
-      <c r="C82" s="36"/>
+      <c r="C82" s="26"/>
       <c r="D82" s="10"/>
     </row>
     <row r="83" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B83" s="18"/>
-      <c r="C83" s="36"/>
+      <c r="C83" s="26"/>
       <c r="D83" s="10"/>
     </row>
     <row r="84" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B84" s="18"/>
-      <c r="C84" s="36"/>
+      <c r="C84" s="26"/>
       <c r="D84" s="10"/>
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B85" s="18"/>
-      <c r="C85" s="41"/>
+      <c r="C85" s="26"/>
       <c r="D85" s="10"/>
     </row>
     <row r="86" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B86" s="18"/>
-      <c r="C86" s="41"/>
+      <c r="C86" s="26"/>
       <c r="D86" s="10"/>
     </row>
     <row r="87" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B87" s="18"/>
-      <c r="C87" s="41"/>
+      <c r="C87" s="26"/>
       <c r="D87" s="10"/>
     </row>
     <row r="88" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B88" s="18"/>
-      <c r="C88" s="41"/>
+      <c r="C88" s="26"/>
       <c r="D88" s="10"/>
     </row>
     <row r="89" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B89" s="18"/>
-      <c r="C89" s="40"/>
+      <c r="C89" s="25"/>
       <c r="D89" s="10"/>
     </row>
     <row r="90" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B90" s="18"/>
-      <c r="C90" s="40"/>
+      <c r="C90" s="25"/>
       <c r="D90" s="10"/>
     </row>
-    <row r="91" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B91" s="22"/>
-      <c r="C91" s="45"/>
-      <c r="D91" s="11"/>
+    <row r="91" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B91" s="18"/>
+      <c r="C91" s="25"/>
+      <c r="D91" s="10"/>
+    </row>
+    <row r="92" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B92" s="18"/>
+      <c r="C92" s="30"/>
+      <c r="D92" s="10"/>
+    </row>
+    <row r="93" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B93" s="18"/>
+      <c r="C93" s="30"/>
+      <c r="D93" s="10"/>
+    </row>
+    <row r="94" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B94" s="18"/>
+      <c r="C94" s="30"/>
+      <c r="D94" s="10"/>
+    </row>
+    <row r="95" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B95" s="18"/>
+      <c r="C95" s="30"/>
+      <c r="D95" s="10"/>
+    </row>
+    <row r="96" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B96" s="18"/>
+      <c r="C96" s="29"/>
+      <c r="D96" s="10"/>
+    </row>
+    <row r="97" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B97" s="18"/>
+      <c r="C97" s="29"/>
+      <c r="D97" s="10"/>
+    </row>
+    <row r="98" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B98" s="22"/>
+      <c r="C98" s="34"/>
+      <c r="D98" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B29:D29"/>
     <mergeCell ref="B3:D3"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
2026 09 10 002
..
</commit_message>
<xml_diff>
--- a/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
+++ b/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58DAE065-B991-4603-BE81-EDC3BC7CB7AC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCE174E0-EFA5-43BD-829F-465BA1A577E7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="8910" windowHeight="10470" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="644">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="646">
   <si>
     <t>내용</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2026,6 +2026,66 @@
   </si>
   <si>
     <t>z축 속도 별도 셋팅. 80% 속도, 20% 속도</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>조그 인터락.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. FMS 오류는 수동 조그 인터락에서 제외
+2. Source Centering 공통 인터락 제거
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. X/Y는 Z==0 대신 설정 가능한 안전 높이와 허용 오차 사용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+4. Z DOWN일 때만 현재 X/Y 영역에 해당하는 Source/Target Centering 확인
+5. 리밋 방향으로는 금지하되 반대쪽 탈출 방향은 허용
+6. 모든 조그 조건을 CanStartManualJog(axis, direction) 하나로 통합
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>7. 조그 상태를 Mouse Up까지 유지하고 CC-Link, BUFFER, Safety, EMS를 계속 감시
+8. 조그 최대 유지시간을 두어 Mouse Up 누락 시 자동 정지. 
+9. 타겟트레이, 소스트레이 내에서 조그인터락 별도 적용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. (z축 이동시 센터링)</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2363,7 +2423,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -2443,9 +2503,6 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="2"/>
-    </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="2"/>
     </xf>
@@ -2453,9 +2510,6 @@
       <alignment horizontal="left" indent="2"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2488,17 +2542,38 @@
     <xf numFmtId="176" fontId="3" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="2"/>
+      <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2790,12 +2865,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
     </row>
     <row r="3" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2813,12 +2888,12 @@
       </c>
     </row>
     <row r="5" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="39"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="37"/>
     </row>
     <row r="6" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="13" t="s">
@@ -2892,12 +2967,12 @@
       <c r="H13" s="12"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="36" t="s">
+      <c r="B16" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="36"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="34"/>
     </row>
     <row r="17" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="18" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2960,13 +3035,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B66418C2-2F25-4DF5-AD93-3985FBAF3208}">
-  <dimension ref="B1:D98"/>
+  <dimension ref="B1:D101"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="9.875" style="20" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="102.375" style="23" customWidth="1"/>
-    <col min="4" max="4" width="68.625" style="8" customWidth="1"/>
+    <col min="4" max="4" width="72.375" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -2982,17 +3057,17 @@
       </c>
     </row>
     <row r="3" spans="2:4" ht="25.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="41" t="s">
         <v>620</v>
       </c>
-      <c r="C3" s="44"/>
-      <c r="D3" s="45"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="43"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="18" t="s">
         <v>617</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="C4" s="49" t="s">
         <v>621</v>
       </c>
       <c r="D4" s="10"/>
@@ -3001,7 +3076,7 @@
       <c r="B5" s="18" t="s">
         <v>617</v>
       </c>
-      <c r="C5" s="46" t="s">
+      <c r="C5" s="50" t="s">
         <v>622</v>
       </c>
       <c r="D5" s="10"/>
@@ -3010,7 +3085,7 @@
       <c r="B6" s="18" t="s">
         <v>617</v>
       </c>
-      <c r="C6" s="31" t="s">
+      <c r="C6" s="51" t="s">
         <v>623</v>
       </c>
       <c r="D6" s="15"/>
@@ -3019,7 +3094,7 @@
       <c r="B7" s="18" t="s">
         <v>624</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="C7" s="52" t="s">
         <v>625</v>
       </c>
       <c r="D7" s="15"/>
@@ -3028,7 +3103,7 @@
       <c r="B8" s="18" t="s">
         <v>626</v>
       </c>
-      <c r="C8" s="31" t="s">
+      <c r="C8" s="51" t="s">
         <v>627</v>
       </c>
       <c r="D8" s="15"/>
@@ -3037,7 +3112,7 @@
       <c r="B9" s="18" t="s">
         <v>629</v>
       </c>
-      <c r="C9" s="31" t="s">
+      <c r="C9" s="51" t="s">
         <v>628</v>
       </c>
       <c r="D9" s="10"/>
@@ -3046,7 +3121,7 @@
       <c r="B10" s="18" t="s">
         <v>630</v>
       </c>
-      <c r="C10" s="31" t="s">
+      <c r="C10" s="51" t="s">
         <v>631</v>
       </c>
       <c r="D10" s="16"/>
@@ -3055,7 +3130,7 @@
       <c r="B11" s="18" t="s">
         <v>632</v>
       </c>
-      <c r="C11" s="31" t="s">
+      <c r="C11" s="51" t="s">
         <v>633</v>
       </c>
       <c r="D11" s="15"/>
@@ -3064,14 +3139,14 @@
       <c r="B12" s="18" t="s">
         <v>634</v>
       </c>
-      <c r="C12" s="31" t="s">
+      <c r="C12" s="51" t="s">
         <v>635</v>
       </c>
       <c r="D12" s="15"/>
     </row>
     <row r="13" spans="2:4" ht="26.25" x14ac:dyDescent="0.3">
       <c r="B13" s="18"/>
-      <c r="C13" s="49" t="s">
+      <c r="C13" s="44" t="s">
         <v>637</v>
       </c>
       <c r="D13" s="10"/>
@@ -3080,7 +3155,7 @@
       <c r="B14" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="C14" s="47" t="s">
+      <c r="C14" s="53" t="s">
         <v>638</v>
       </c>
       <c r="D14" s="10"/>
@@ -3089,7 +3164,7 @@
       <c r="B15" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="C15" s="47" t="s">
+      <c r="C15" s="53" t="s">
         <v>639</v>
       </c>
       <c r="D15" s="10"/>
@@ -3098,7 +3173,7 @@
       <c r="B16" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="C16" s="47" t="s">
+      <c r="C16" s="53" t="s">
         <v>640</v>
       </c>
       <c r="D16" s="10"/>
@@ -3107,7 +3182,7 @@
       <c r="B17" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="C17" s="48" t="s">
+      <c r="C17" s="54" t="s">
         <v>642</v>
       </c>
       <c r="D17" s="10"/>
@@ -3116,7 +3191,7 @@
       <c r="B18" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="C18" s="47" t="s">
+      <c r="C18" s="53" t="s">
         <v>641</v>
       </c>
       <c r="D18" s="10"/>
@@ -3125,15 +3200,21 @@
       <c r="B19" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="C19" s="47" t="s">
+      <c r="C19" s="53" t="s">
         <v>643</v>
       </c>
       <c r="D19" s="10"/>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B20" s="18"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="10"/>
+    <row r="20" spans="2:4" s="47" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
+      <c r="B20" s="45" t="s">
+        <v>636</v>
+      </c>
+      <c r="C20" s="48" t="s">
+        <v>644</v>
+      </c>
+      <c r="D20" s="46" t="s">
+        <v>645</v>
+      </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B21" s="18"/>
@@ -3152,104 +3233,104 @@
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B24" s="18"/>
-      <c r="C24" s="29"/>
+      <c r="C24" s="28"/>
       <c r="D24" s="10"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B25" s="18"/>
-      <c r="C25" s="29"/>
+      <c r="C25" s="28"/>
       <c r="D25" s="10"/>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B26" s="18"/>
-      <c r="C26" s="29"/>
+      <c r="C26" s="28"/>
       <c r="D26" s="10"/>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B27" s="18"/>
-      <c r="C27" s="28"/>
+      <c r="C27" s="29"/>
       <c r="D27" s="10"/>
     </row>
-    <row r="28" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B28" s="18"/>
-      <c r="C28" s="30"/>
+      <c r="C28" s="29"/>
       <c r="D28" s="10"/>
     </row>
-    <row r="29" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="40" t="s">
-        <v>619</v>
-      </c>
-      <c r="C29" s="41"/>
-      <c r="D29" s="42"/>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B29" s="18"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="10"/>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B30" s="18"/>
-      <c r="C30" s="32"/>
+      <c r="C30" s="28"/>
       <c r="D30" s="10"/>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B31" s="18"/>
-      <c r="C31" s="33"/>
+      <c r="C31" s="30"/>
       <c r="D31" s="10"/>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B32" s="18"/>
-      <c r="C32" s="32"/>
-      <c r="D32" s="10"/>
+    <row r="32" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B32" s="38" t="s">
+        <v>619</v>
+      </c>
+      <c r="C32" s="39"/>
+      <c r="D32" s="40"/>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B33" s="18"/>
-      <c r="C33" s="33"/>
+      <c r="C33" s="31"/>
       <c r="D33" s="10"/>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B34" s="18"/>
-      <c r="C34" s="33"/>
+      <c r="C34" s="32"/>
       <c r="D34" s="10"/>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B35" s="18"/>
-      <c r="C35" s="33"/>
+      <c r="C35" s="31"/>
       <c r="D35" s="10"/>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B36" s="18"/>
-      <c r="C36" s="33"/>
+      <c r="C36" s="32"/>
       <c r="D36" s="10"/>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B37" s="18"/>
-      <c r="C37" s="33"/>
+      <c r="C37" s="32"/>
       <c r="D37" s="10"/>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B38" s="18"/>
-      <c r="C38" s="33"/>
+      <c r="C38" s="32"/>
       <c r="D38" s="10"/>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B39" s="18"/>
-      <c r="C39" s="33"/>
+      <c r="C39" s="32"/>
       <c r="D39" s="10"/>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B40" s="18"/>
-      <c r="C40" s="33"/>
+      <c r="C40" s="32"/>
       <c r="D40" s="10"/>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B41" s="18"/>
-      <c r="C41" s="33"/>
+      <c r="C41" s="32"/>
       <c r="D41" s="10"/>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B42" s="18"/>
-      <c r="C42" s="33"/>
+      <c r="C42" s="32"/>
       <c r="D42" s="10"/>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B43" s="18"/>
-      <c r="C43" s="33"/>
+      <c r="C43" s="32"/>
       <c r="D43" s="10"/>
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.3">
@@ -3269,77 +3350,77 @@
     </row>
     <row r="47" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B47" s="18"/>
-      <c r="C47" s="33"/>
+      <c r="C47" s="31"/>
       <c r="D47" s="10"/>
     </row>
     <row r="48" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B48" s="18"/>
-      <c r="C48" s="33"/>
+      <c r="C48" s="31"/>
       <c r="D48" s="10"/>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B49" s="18"/>
-      <c r="C49" s="32"/>
+      <c r="C49" s="31"/>
       <c r="D49" s="10"/>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B50" s="18"/>
-      <c r="C50" s="33"/>
+      <c r="C50" s="32"/>
       <c r="D50" s="10"/>
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B51" s="18"/>
-      <c r="C51" s="29"/>
+      <c r="C51" s="32"/>
       <c r="D51" s="10"/>
     </row>
     <row r="52" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B52" s="18"/>
-      <c r="C52" s="29"/>
+      <c r="C52" s="31"/>
       <c r="D52" s="10"/>
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B53" s="18"/>
-      <c r="C53" s="33"/>
+      <c r="C53" s="32"/>
       <c r="D53" s="10"/>
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B54" s="18"/>
-      <c r="C54" s="33"/>
+      <c r="C54" s="29"/>
       <c r="D54" s="10"/>
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B55" s="18"/>
-      <c r="C55" s="33"/>
+      <c r="C55" s="29"/>
       <c r="D55" s="10"/>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B56" s="18"/>
-      <c r="C56" s="33"/>
+      <c r="C56" s="32"/>
       <c r="D56" s="10"/>
     </row>
     <row r="57" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B57" s="18"/>
-      <c r="C57" s="33"/>
+      <c r="C57" s="32"/>
       <c r="D57" s="10"/>
     </row>
     <row r="58" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B58" s="18"/>
-      <c r="C58" s="33"/>
+      <c r="C58" s="32"/>
       <c r="D58" s="10"/>
     </row>
     <row r="59" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B59" s="18"/>
-      <c r="C59" s="33"/>
+      <c r="C59" s="32"/>
       <c r="D59" s="10"/>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B60" s="18"/>
-      <c r="C60" s="29"/>
+      <c r="C60" s="32"/>
       <c r="D60" s="10"/>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B61" s="18"/>
-      <c r="C61" s="33"/>
+      <c r="C61" s="32"/>
       <c r="D61" s="10"/>
     </row>
     <row r="62" spans="2:4" x14ac:dyDescent="0.3">
@@ -3354,12 +3435,12 @@
     </row>
     <row r="64" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B64" s="18"/>
-      <c r="C64" s="33"/>
+      <c r="C64" s="32"/>
       <c r="D64" s="10"/>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B65" s="18"/>
-      <c r="C65" s="29"/>
+      <c r="C65" s="31"/>
       <c r="D65" s="10"/>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.3">
@@ -3369,57 +3450,57 @@
     </row>
     <row r="67" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B67" s="18"/>
-      <c r="C67" s="28"/>
+      <c r="C67" s="32"/>
       <c r="D67" s="10"/>
     </row>
     <row r="68" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B68" s="18"/>
-      <c r="C68" s="26"/>
-      <c r="D68" s="17"/>
+      <c r="C68" s="29"/>
+      <c r="D68" s="10"/>
     </row>
     <row r="69" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B69" s="18"/>
-      <c r="C69" s="33"/>
+      <c r="C69" s="29"/>
       <c r="D69" s="10"/>
     </row>
     <row r="70" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B70" s="18"/>
-      <c r="C70" s="33"/>
+      <c r="C70" s="28"/>
       <c r="D70" s="10"/>
     </row>
     <row r="71" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B71" s="18"/>
-      <c r="C71" s="33"/>
-      <c r="D71" s="10"/>
+      <c r="C71" s="26"/>
+      <c r="D71" s="17"/>
     </row>
     <row r="72" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B72" s="18"/>
-      <c r="C72" s="33"/>
+      <c r="C72" s="32"/>
       <c r="D72" s="10"/>
     </row>
     <row r="73" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B73" s="18"/>
-      <c r="C73" s="33"/>
+      <c r="C73" s="32"/>
       <c r="D73" s="10"/>
     </row>
     <row r="74" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B74" s="18"/>
-      <c r="C74" s="26"/>
+      <c r="C74" s="32"/>
       <c r="D74" s="10"/>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B75" s="18"/>
-      <c r="C75" s="33"/>
+      <c r="C75" s="32"/>
       <c r="D75" s="10"/>
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B76" s="18"/>
-      <c r="C76" s="26"/>
+      <c r="C76" s="32"/>
       <c r="D76" s="10"/>
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B77" s="18"/>
-      <c r="C77" s="32"/>
+      <c r="C77" s="26"/>
       <c r="D77" s="10"/>
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.3">
@@ -3434,12 +3515,12 @@
     </row>
     <row r="80" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B80" s="18"/>
-      <c r="C80" s="26"/>
+      <c r="C80" s="31"/>
       <c r="D80" s="10"/>
     </row>
     <row r="81" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B81" s="18"/>
-      <c r="C81" s="26"/>
+      <c r="C81" s="31"/>
       <c r="D81" s="10"/>
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.3">
@@ -3479,32 +3560,32 @@
     </row>
     <row r="89" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B89" s="18"/>
-      <c r="C89" s="25"/>
+      <c r="C89" s="26"/>
       <c r="D89" s="10"/>
     </row>
     <row r="90" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B90" s="18"/>
-      <c r="C90" s="25"/>
+      <c r="C90" s="26"/>
       <c r="D90" s="10"/>
     </row>
     <row r="91" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B91" s="18"/>
-      <c r="C91" s="25"/>
+      <c r="C91" s="26"/>
       <c r="D91" s="10"/>
     </row>
     <row r="92" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B92" s="18"/>
-      <c r="C92" s="30"/>
+      <c r="C92" s="25"/>
       <c r="D92" s="10"/>
     </row>
     <row r="93" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B93" s="18"/>
-      <c r="C93" s="30"/>
+      <c r="C93" s="25"/>
       <c r="D93" s="10"/>
     </row>
     <row r="94" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B94" s="18"/>
-      <c r="C94" s="30"/>
+      <c r="C94" s="25"/>
       <c r="D94" s="10"/>
     </row>
     <row r="95" spans="2:4" x14ac:dyDescent="0.3">
@@ -3514,22 +3595,37 @@
     </row>
     <row r="96" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B96" s="18"/>
-      <c r="C96" s="29"/>
+      <c r="C96" s="30"/>
       <c r="D96" s="10"/>
     </row>
     <row r="97" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B97" s="18"/>
-      <c r="C97" s="29"/>
+      <c r="C97" s="30"/>
       <c r="D97" s="10"/>
     </row>
-    <row r="98" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B98" s="22"/>
-      <c r="C98" s="34"/>
-      <c r="D98" s="11"/>
+    <row r="98" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B98" s="18"/>
+      <c r="C98" s="30"/>
+      <c r="D98" s="10"/>
+    </row>
+    <row r="99" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B99" s="18"/>
+      <c r="C99" s="29"/>
+      <c r="D99" s="10"/>
+    </row>
+    <row r="100" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B100" s="18"/>
+      <c r="C100" s="29"/>
+      <c r="D100" s="10"/>
+    </row>
+    <row r="101" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B101" s="22"/>
+      <c r="C101" s="33"/>
+      <c r="D101" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B32:D32"/>
     <mergeCell ref="B3:D3"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>